<commit_message>
Odd-nominal fallback rule for even-ladder dead zones (GRC102501/1 -> THC7)
Management rule addition: an isolated result that no even nominal can hold
within +/-10% takes the adjacent ODD whole-number nominal instead, formed
without overlap against neighbouring ranges. Resolves the one dead-zone
exception: GRC102501/1 (7.05, declared) -> GRC_THC7:CBD1, 6.30-7.70,
full +/-10%. All 85 batches now placed across 52 grades; zero exceptions.
Even nominals remain the default; the fallback fires only when the even
ladder mathematically refuses (dead zones 6.61-7.19 and 8.81-8.99).

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/potency_study/ImB_Potency_Grade_Ranges.xlsx
+++ b/deliverables/potency_study/ImB_Potency_Grade_Ranges.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1747,299 +1747,291 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>GRC_THC7 : CBD1</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_GRC-II</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10% — ODD nominal (fallback rule 5)</t>
+        </is>
+      </c>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>GRC102501/1 7.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>High Pro Amnesia</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>HPA</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>HPA_THC22 : CBD1</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_HPA-I</t>
         </is>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="F32" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="G32" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="H31" s="6" t="n">
+      <c r="H32" s="6" t="n">
         <v>24.2</v>
       </c>
-      <c r="I31" s="6" t="n">
+      <c r="I32" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K31" s="8" t="inlineStr">
+      <c r="K32" s="8" t="inlineStr">
         <is>
           <t>HPA1024_01 21.61, HPA052501 20.39</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr"/>
-      <c r="C32" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>HPA_THC18 : CBD1</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_HPA-II</t>
         </is>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="F33" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="G32" s="6" t="n">
+      <c r="G33" s="6" t="n">
         <v>16.2</v>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H33" s="6" t="n">
         <v>19.79</v>
       </c>
-      <c r="I32" s="6" t="n">
+      <c r="I33" s="6" t="n">
         <v>3.59</v>
       </c>
-      <c r="J32" s="9" t="inlineStr">
+      <c r="J33" s="9" t="inlineStr">
         <is>
           <t>clipped (no-overlap rule)</t>
         </is>
       </c>
-      <c r="K32" s="8" t="inlineStr">
+      <c r="K33" s="8" t="inlineStr">
         <is>
           <t>HPA1024 17.31</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Jelly Donutz</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>JD</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>JD_THC20 : CBD1</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_JD-I</t>
         </is>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="F34" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G33" s="6" t="n">
+      <c r="G34" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="H34" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="I33" s="6" t="n">
+      <c r="I34" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="J33" s="7" t="inlineStr">
+      <c r="J34" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K33" s="8" t="inlineStr">
+      <c r="K34" s="8" t="inlineStr">
         <is>
           <t>JD012603/02 20.54, JD112501 20.32, JD022601 18.58, JD012601 18.16</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>JD_THC16 : CBD1</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_JD-II</t>
         </is>
       </c>
-      <c r="F34" s="6" t="n">
+      <c r="F35" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="G34" s="6" t="n">
+      <c r="G35" s="6" t="n">
         <v>14.4</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H35" s="6" t="n">
         <v>17.6</v>
       </c>
-      <c r="I34" s="6" t="n">
+      <c r="I35" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="J34" s="7" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K34" s="8" t="inlineStr">
+      <c r="K35" s="8" t="inlineStr">
         <is>
           <t>JD012603/01 16.71, JD012603/02V 15.16</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Jokerz 31</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>J31</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>J31_THC22 : CBD1</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_J31-I</t>
         </is>
       </c>
-      <c r="F35" s="6" t="n">
+      <c r="F36" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G35" s="6" t="n">
+      <c r="G36" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="H35" s="6" t="n">
+      <c r="H36" s="6" t="n">
         <v>24.2</v>
       </c>
-      <c r="I35" s="6" t="n">
+      <c r="I36" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="J35" s="7" t="inlineStr">
+      <c r="J36" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K35" s="8" t="inlineStr">
+      <c r="K36" s="8" t="inlineStr">
         <is>
           <t>J31122501 21.84, J31112501 20.21</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr"/>
-      <c r="C36" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>J31_THC18 : CBD1</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_J31-II</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="G36" s="6" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="H36" s="6" t="n">
-        <v>19.79</v>
-      </c>
-      <c r="I36" s="6" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="J36" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K36" s="8" t="inlineStr">
-        <is>
-          <t>J31102501 17.32</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Kush Crasher</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>KC</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>KC_THC18 : CBD1</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_KC-I</t>
         </is>
       </c>
       <c r="F37" s="6" t="n">
@@ -2049,31 +2041,31 @@
         <v>16.2</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>19.8</v>
+        <v>19.79</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>3.59</v>
+      </c>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>clipped (no-overlap rule)</t>
         </is>
       </c>
       <c r="K37" s="8" t="inlineStr">
         <is>
-          <t>KC102501 17.04</t>
+          <t>J31102501 17.32</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Motor Breath</t>
+          <t>Kush Crasher</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -2083,165 +2075,173 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>MB_THC18 : CBD1</t>
+          <t>KC_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_MB-I</t>
+          <t>QCSP_001_KC-I</t>
         </is>
       </c>
       <c r="F38" s="6" t="n">
         <v>18</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>16.83</v>
+        <v>16.2</v>
       </c>
       <c r="H38" s="6" t="n">
         <v>19.8</v>
       </c>
       <c r="I38" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K38" s="8" t="inlineStr">
+        <is>
+          <t>KC102501 17.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Motor Breath</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>MB_THC18 : CBD1</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_MB-I</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>16.83</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="I39" s="6" t="n">
         <v>2.97</v>
       </c>
-      <c r="J38" s="9" t="inlineStr">
+      <c r="J39" s="9" t="inlineStr">
         <is>
           <t>clipped (no-overlap rule)</t>
         </is>
       </c>
-      <c r="K38" s="8" t="inlineStr">
+      <c r="K39" s="8" t="inlineStr">
         <is>
           <t>MB0824_04 18.67</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr"/>
-      <c r="B39" s="5" t="inlineStr"/>
-      <c r="C39" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr"/>
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>MB_THC16 : CBD1</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_MB-II</t>
         </is>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="F40" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G40" s="6" t="n">
         <v>14.4</v>
       </c>
-      <c r="H39" s="6" t="n">
+      <c r="H40" s="6" t="n">
         <v>16.82</v>
       </c>
-      <c r="I39" s="6" t="n">
+      <c r="I40" s="6" t="n">
         <v>2.42</v>
       </c>
-      <c r="J39" s="9" t="inlineStr">
+      <c r="J40" s="9" t="inlineStr">
         <is>
           <t>clipped (no-overlap rule)</t>
         </is>
       </c>
-      <c r="K39" s="8" t="inlineStr">
+      <c r="K40" s="8" t="inlineStr">
         <is>
           <t>MB0824_05 16.82</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Orange Punch Mimosa</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>OPM</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>OPM_THC22 : CBD1</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_OPM-I</t>
         </is>
       </c>
-      <c r="F40" s="6" t="n">
+      <c r="F41" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="G41" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="H40" s="6" t="n">
+      <c r="H41" s="6" t="n">
         <v>24.2</v>
       </c>
-      <c r="I40" s="6" t="n">
+      <c r="I41" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="J40" s="7" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K40" s="8" t="inlineStr">
+      <c r="K41" s="8" t="inlineStr">
         <is>
           <t>OPM1024 20.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr"/>
-      <c r="B41" s="5" t="inlineStr"/>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>II</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>OPM_THC18 : CBD1</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_OPM-II</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="G41" s="6" t="n">
-        <v>16.56</v>
-      </c>
-      <c r="H41" s="6" t="n">
-        <v>19.79</v>
-      </c>
-      <c r="I41" s="6" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="J41" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="inlineStr">
-        <is>
-          <t>OPM1024_02 18.04</t>
         </is>
       </c>
     </row>
@@ -2250,30 +2250,30 @@
       <c r="B42" s="5" t="inlineStr"/>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC16 : CBD1</t>
+          <t>OPM_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-III</t>
+          <t>QCSP_001_OPM-II</t>
         </is>
       </c>
       <c r="F42" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>14.4</v>
+        <v>16.56</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>16.55</v>
+        <v>19.79</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>2.15</v>
+        <v>3.23</v>
       </c>
       <c r="J42" s="9" t="inlineStr">
         <is>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>OPM1024_03 16.55, OMP1024_01 15.38</t>
+          <t>OPM1024_02 18.04</t>
         </is>
       </c>
     </row>
@@ -2291,30 +2291,30 @@
       <c r="B43" s="5" t="inlineStr"/>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC14 : CBD1</t>
+          <t>OPM_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-IV</t>
+          <t>QCSP_001_OPM-III</t>
         </is>
       </c>
       <c r="F43" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>12.6</v>
+        <v>14.4</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>14.39</v>
+        <v>16.55</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>1.79</v>
+        <v>2.15</v>
       </c>
       <c r="J43" s="9" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>OPM052501 14.16</t>
+          <t>OPM1024_03 16.55, OMP1024_01 15.38</t>
         </is>
       </c>
     </row>
@@ -2332,39 +2332,39 @@
       <c r="B44" s="5" t="inlineStr"/>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC10 : CBD1</t>
+          <t>OPM_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-V</t>
+          <t>QCSP_001_OPM-IV</t>
         </is>
       </c>
       <c r="F44" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>9</v>
+        <v>12.6</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>11</v>
+        <v>14.39</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J44" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>1.79</v>
+      </c>
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t>clipped (no-overlap rule)</t>
         </is>
       </c>
       <c r="K44" s="8" t="inlineStr">
         <is>
-          <t>OPM092501 9.43</t>
+          <t>OPM052501 14.16</t>
         </is>
       </c>
     </row>
@@ -2373,129 +2373,129 @@
       <c r="B45" s="5" t="inlineStr"/>
       <c r="C45" s="5" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>OPM_THC10 : CBD1</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_OPM-V</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K45" s="8" t="inlineStr">
+        <is>
+          <t>OPM092501 9.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr"/>
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
           <t>VI</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>OPM_THC8 : CBD1</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_OPM-VI</t>
         </is>
       </c>
-      <c r="F45" s="6" t="n">
+      <c r="F46" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G45" s="6" t="n">
+      <c r="G46" s="6" t="n">
         <v>7.2</v>
       </c>
-      <c r="H45" s="6" t="n">
+      <c r="H46" s="6" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="I45" s="6" t="n">
+      <c r="I46" s="6" t="n">
         <v>1.6</v>
       </c>
-      <c r="J45" s="7" t="inlineStr">
+      <c r="J46" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K45" s="8" t="inlineStr">
+      <c r="K46" s="8" t="inlineStr">
         <is>
           <t>OPM112501 8.00, OPM122501 7.91</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Permanent Marker</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>PM_THC14 : CBD1</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_PM-I</t>
         </is>
       </c>
-      <c r="F46" s="6" t="n">
+      <c r="F47" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="G46" s="6" t="n">
+      <c r="G47" s="6" t="n">
         <v>12.6</v>
       </c>
-      <c r="H46" s="6" t="n">
+      <c r="H47" s="6" t="n">
         <v>15.4</v>
       </c>
-      <c r="I46" s="6" t="n">
+      <c r="I47" s="6" t="n">
         <v>2.8</v>
       </c>
-      <c r="J46" s="7" t="inlineStr">
+      <c r="J47" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K46" s="8" t="inlineStr">
+      <c r="K47" s="8" t="inlineStr">
         <is>
           <t>PM112501 13.33</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr"/>
-      <c r="B47" s="5" t="inlineStr"/>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>II</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>PM_THC12 : CBD1</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_PM-II</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="G47" s="6" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="H47" s="6" t="n">
-        <v>12.59</v>
-      </c>
-      <c r="I47" s="6" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="J47" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K47" s="8" t="inlineStr">
-        <is>
-          <t>PM092501 12.25</t>
         </is>
       </c>
     </row>
@@ -2504,27 +2504,27 @@
       <c r="B48" s="5" t="inlineStr"/>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>PM_THC10 : CBD1</t>
+          <t>PM_THC12 : CBD1</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_PM-III</t>
+          <t>QCSP_001_PM-II</t>
         </is>
       </c>
       <c r="F48" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>9</v>
+        <v>10.8</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>10.79</v>
+        <v>12.59</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>1.79</v>
@@ -2536,297 +2536,289 @@
       </c>
       <c r="K48" s="8" t="inlineStr">
         <is>
+          <t>PM092501 12.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>PM_THC10 : CBD1</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_PM-III</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="I49" s="6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>clipped (no-overlap rule)</t>
+        </is>
+      </c>
+      <c r="K49" s="8" t="inlineStr">
+        <is>
           <t>PM072501 10.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>Pure Michigen</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>PUM</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>PUM_THC16 : CBD1</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_PUM-I</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="G49" s="6" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H49" s="6" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="I49" s="6" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="J49" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
-        </is>
-      </c>
-      <c r="K49" s="8" t="inlineStr">
-        <is>
-          <t>PUM102501 15.63</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
+          <t>Pure Michigen</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>PUM</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>PUM_THC16 : CBD1</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_PUM-I</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K50" s="8" t="inlineStr">
+        <is>
+          <t>PUM102501 15.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
           <t>Scrambler</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>SCR</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>SCR_THC22 : CBD1</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_SCR-I</t>
         </is>
       </c>
-      <c r="F50" s="6" t="n">
+      <c r="F51" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G50" s="6" t="n">
+      <c r="G51" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="H50" s="6" t="n">
+      <c r="H51" s="6" t="n">
         <v>24.2</v>
       </c>
-      <c r="I50" s="6" t="n">
+      <c r="I51" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="J50" s="7" t="inlineStr">
+      <c r="J51" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K50" s="8" t="inlineStr">
+      <c r="K51" s="8" t="inlineStr">
         <is>
           <t>SCR022601 21.92</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr"/>
-      <c r="B51" s="5" t="inlineStr"/>
-      <c r="C51" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr"/>
+      <c r="B52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>SCR_THC18 : CBD1</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_SCR-II</t>
         </is>
       </c>
-      <c r="F51" s="6" t="n">
+      <c r="F52" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="G51" s="6" t="n">
+      <c r="G52" s="6" t="n">
         <v>16.2</v>
       </c>
-      <c r="H51" s="6" t="n">
+      <c r="H52" s="6" t="n">
         <v>19.79</v>
       </c>
-      <c r="I51" s="6" t="n">
+      <c r="I52" s="6" t="n">
         <v>3.59</v>
       </c>
-      <c r="J51" s="9" t="inlineStr">
+      <c r="J52" s="9" t="inlineStr">
         <is>
           <t>clipped (no-overlap rule)</t>
         </is>
       </c>
-      <c r="K51" s="8" t="inlineStr">
+      <c r="K52" s="8" t="inlineStr">
         <is>
           <t>SCR012601 18.07, SCR012603 17.84, SCR112501 17.13</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>Sleepy Joy</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>SJ</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>SJ_THC12 : CBD1</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_SJ-I</t>
         </is>
       </c>
-      <c r="F52" s="6" t="n">
+      <c r="F53" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="G52" s="6" t="n">
+      <c r="G53" s="6" t="n">
         <v>10.97</v>
       </c>
-      <c r="H52" s="6" t="n">
+      <c r="H53" s="6" t="n">
         <v>13.2</v>
       </c>
-      <c r="I52" s="6" t="n">
+      <c r="I53" s="6" t="n">
         <v>2.23</v>
       </c>
-      <c r="J52" s="9" t="inlineStr">
+      <c r="J53" s="9" t="inlineStr">
         <is>
           <t>clipped (no-overlap rule)</t>
         </is>
       </c>
-      <c r="K52" s="8" t="inlineStr">
+      <c r="K53" s="8" t="inlineStr">
         <is>
           <t>SJ102501 11.20</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr"/>
-      <c r="B53" s="5" t="inlineStr"/>
-      <c r="C53" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr"/>
+      <c r="B54" s="5" t="inlineStr"/>
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>SJ_THC10 : CBD1</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_SJ-II</t>
         </is>
       </c>
-      <c r="F53" s="6" t="n">
+      <c r="F54" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G53" s="6" t="n">
+      <c r="G54" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H53" s="6" t="n">
+      <c r="H54" s="6" t="n">
         <v>10.96</v>
       </c>
-      <c r="I53" s="6" t="n">
+      <c r="I54" s="6" t="n">
         <v>1.96</v>
       </c>
-      <c r="J53" s="9" t="inlineStr">
+      <c r="J54" s="9" t="inlineStr">
         <is>
           <t>clipped (no-overlap rule)</t>
         </is>
       </c>
-      <c r="K53" s="8" t="inlineStr">
+      <c r="K54" s="8" t="inlineStr">
         <is>
           <t>SJ092501 10.96, SJ112501 9.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Wedding Cake</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>WED</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>WED_THC22 : CBD1</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_WED-I</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="I54" s="6" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J54" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
-        </is>
-      </c>
-      <c r="K54" s="8" t="inlineStr">
-        <is>
-          <t>WED102501 22.05</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Wedding Crasher</t>
+          <t>Wedding Cake</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -2836,12 +2828,12 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>WC_THC22 : CBD1</t>
+          <t>WED_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_WC-I</t>
+          <t>QCSP_001_WED-I</t>
         </is>
       </c>
       <c r="F55" s="6" t="n">
@@ -2862,6 +2854,55 @@
         </is>
       </c>
       <c r="K55" s="8" t="inlineStr">
+        <is>
+          <t>WED102501 22.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Wedding Crasher</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>WC_THC22 : CBD1</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_WC-I</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K56" s="8" t="inlineStr">
         <is>
           <t>WC072501 22.11, WC082501 21.67</t>
         </is>
@@ -2878,7 +2919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4728,43 +4769,47 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>HPA1024_01</t>
+          <t>GRC102501/1</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>High Pro Amnesia</t>
+          <t>Graps &amp; Creme</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>HPA_THC22 : CBD1</t>
+          <t>GRC_THC7 : CBD1</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>21.61</v>
+        <v>7.05</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>197-14-К/26, 07.08.2026, FARM</t>
+          <t>owner-declared value</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H49" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>declared value — no eCoA yet, grade provisional until tested</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>HPA052501</t>
+          <t>HPA1024_01</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
@@ -4783,11 +4828,11 @@
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>20.39</v>
+        <v>21.61</v>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>ППК25278, 19.09.2025, UKIM</t>
+          <t>197-14-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -4800,7 +4845,7 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>HPA1024</t>
+          <t>HPA052501</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -4810,20 +4855,20 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>HPA_THC18 : CBD1</t>
+          <t>HPA_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>17.31</v>
+        <v>20.39</v>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>197-13-К/26, 07.08.2026, FARM</t>
+          <t>ППК25278, 19.09.2025, UKIM</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -4836,30 +4881,30 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>JD012603/02</t>
+          <t>HPA1024</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Jelly Donutz</t>
+          <t>High Pro Amnesia</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>JD_THC20 : CBD1</t>
+          <t>HPA_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>20.54</v>
+        <v>17.31</v>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>ППК26113, 30.06.2026, UKIM</t>
+          <t>197-13-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -4872,7 +4917,7 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>JD112501</t>
+          <t>JD012603/02</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -4891,11 +4936,11 @@
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>20.32</v>
+        <v>20.54</v>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>197-15-К/26, 07.08.2026, FARM</t>
+          <t>ППК26113, 30.06.2026, UKIM</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -4908,7 +4953,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>JD022601</t>
+          <t>JD112501</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
@@ -4927,28 +4972,24 @@
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>18.58</v>
+        <v>20.32</v>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>ППК26115, 30.06.2026, UKIM</t>
+          <t>197-15-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H54" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H54" s="8" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>JD012601</t>
+          <t>JD022601</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -4967,11 +5008,11 @@
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>18.16</v>
+        <v>18.58</v>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>ППК26064, 11.05.2026, UKIM</t>
+          <t>ППК26115, 30.06.2026, UKIM</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -4988,7 +5029,7 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>JD012603/01</t>
+          <t>JD012601</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
@@ -4998,37 +5039,37 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>JD_THC16 : CBD1</t>
+          <t>JD_THC20 : CBD1</t>
         </is>
       </c>
       <c r="E56" s="6" t="n">
-        <v>16.71</v>
+        <v>18.16</v>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>owner-declared value</t>
+          <t>ППК26064, 11.05.2026, UKIM</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>declared value — no eCoA yet, grade provisional until tested</t>
+          <t>code assigned by value (batch not on the tranche list)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>JD012603/02V</t>
+          <t>JD012603/01</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -5047,11 +5088,11 @@
         </is>
       </c>
       <c r="E57" s="6" t="n">
-        <v>15.16</v>
+        <v>16.71</v>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>ППК26111, 30.06.2026, UKIM</t>
+          <t>owner-declared value</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -5059,52 +5100,52 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H57" s="8" t="inlineStr"/>
+      <c r="H57" s="8" t="inlineStr">
+        <is>
+          <t>declared value — no eCoA yet, grade provisional until tested</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>J31122501</t>
+          <t>JD012603/02V</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Jokerz 31</t>
+          <t>Jelly Donutz</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>J31_THC22 : CBD1</t>
+          <t>JD_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E58" s="6" t="n">
-        <v>21.84</v>
+        <v>15.16</v>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>machine-trimmed preparation, CoQ-forming (CoQ-PP-2026-0054); hand-trimmed 19.84 is the experimental prep</t>
+          <t>ППК26111, 30.06.2026, UKIM</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H58" s="8" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>J31112501</t>
+          <t>J31122501</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -5123,11 +5164,11 @@
         </is>
       </c>
       <c r="E59" s="6" t="n">
-        <v>20.21</v>
+        <v>21.84</v>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>100-1-K/26, 09.04.2026, FARM</t>
+          <t>machine-trimmed preparation, CoQ-forming (CoQ-PP-2026-0054); hand-trimmed 19.84 is the experimental prep</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -5144,7 +5185,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>J31102501</t>
+          <t>J31112501</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
@@ -5154,56 +5195,60 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>J31_THC18 : CBD1</t>
+          <t>J31_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>17.32</v>
+        <v>20.21</v>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>197-16-К/26, 07.08.2026, FARM</t>
+          <t>100-1-K/26, 09.04.2026, FARM</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H60" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="8" t="inlineStr">
+        <is>
+          <t>code assigned by value (batch not on the tranche list)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>KC102501</t>
+          <t>J31102501</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Kush Crasher</t>
+          <t>Jokerz 31</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>KC_THC18 : CBD1</t>
+          <t>J31_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>17.04</v>
+        <v>17.32</v>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>051-4-K/26, 04.03.2026, FARM</t>
+          <t>197-16-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -5216,12 +5261,12 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>MB0824_04</t>
+          <t>KC102501</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Motor Breath</t>
+          <t>Kush Crasher</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -5231,32 +5276,28 @@
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>MB_THC18 : CBD1</t>
+          <t>KC_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>18.67</v>
+        <v>17.04</v>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>ППК25118, 06.05.2025, UKIM</t>
+          <t>051-4-K/26, 04.03.2026, FARM</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H62" s="8" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>MB0824_05</t>
+          <t>MB0824_04</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -5266,56 +5307,60 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>MB_THC16 : CBD1</t>
+          <t>MB_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>16.82</v>
+        <v>18.67</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>ППК52211, 28.07.2025, UKIM</t>
+          <t>ППК25118, 06.05.2025, UKIM</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H63" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="8" t="inlineStr">
+        <is>
+          <t>code assigned by value (batch not on the tranche list)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>OPM1024</t>
+          <t>MB0824_05</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Orange Punch Mimosa</t>
+          <t>Motor Breath</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>OPM_THC22 : CBD1</t>
+          <t>MB_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>20.03</v>
+        <v>16.82</v>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>197-17-К/26, 07.08.2026, FARM</t>
+          <t>ППК52211, 28.07.2025, UKIM</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -5328,7 +5373,7 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>OPM1024_02</t>
+          <t>OPM1024</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
@@ -5338,20 +5383,20 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>OPM_THC18 : CBD1</t>
+          <t>OPM_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>18.04</v>
+        <v>20.03</v>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>197-18-К/26, 07.08.2026, FARM</t>
+          <t>197-17-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
@@ -5364,7 +5409,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>OPM1024_03</t>
+          <t>OPM1024_02</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
@@ -5374,20 +5419,20 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>OPM_THC16 : CBD1</t>
+          <t>OPM_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>16.55</v>
+        <v>18.04</v>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>ППК25210, 28.07.2025, UKIM</t>
+          <t>197-18-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
@@ -5400,7 +5445,7 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>OMP1024_01</t>
+          <t>OPM1024_03</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
@@ -5419,11 +5464,11 @@
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>15.38</v>
+        <v>16.55</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>ППК25117, 06.05.2025, UKIM</t>
+          <t>ППК25210, 28.07.2025, UKIM</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
@@ -5436,7 +5481,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>OPM052501</t>
+          <t>OMP1024_01</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
@@ -5446,37 +5491,33 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>OPM_THC14 : CBD1</t>
+          <t>OPM_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>14.16</v>
+        <v>15.38</v>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>ППК52557, 05.09.2025, UKIM</t>
+          <t>ППК25117, 06.05.2025, UKIM</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H68" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H68" s="8" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>OPM092501</t>
+          <t>OPM052501</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
@@ -5486,33 +5527,37 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>OPM_THC10 : CBD1</t>
+          <t>OPM_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>9.43</v>
+        <v>14.16</v>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>ППК26008, 21.01.2026, UKIM</t>
+          <t>ППК52557, 05.09.2025, UKIM</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H69" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="8" t="inlineStr">
+        <is>
+          <t>code assigned by value (batch not on the tranche list)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>OPM112501</t>
+          <t>OPM092501</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
@@ -5522,149 +5567,149 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>VI</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>OPM_THC8 : CBD1</t>
+          <t>OPM_THC10 : CBD1</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>8</v>
+        <v>9.43</v>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>ППК26031, 05.03.2026, UKIM</t>
+          <t>ППК26008, 21.01.2026, UKIM</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H70" s="8" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
+          <t>OPM112501</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>Orange Punch Mimosa</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>OPM_THC8 : CBD1</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>ППК26031, 05.03.2026, UKIM</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
+        <is>
+          <t>code assigned by value (batch not on the tranche list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
           <t>OPM122501</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>Orange Punch Mimosa</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>VI</t>
         </is>
       </c>
-      <c r="D71" s="8" t="inlineStr">
+      <c r="D72" s="8" t="inlineStr">
         <is>
           <t>OPM_THC8 : CBD1</t>
         </is>
       </c>
-      <c r="E71" s="6" t="n">
+      <c r="E72" s="6" t="n">
         <v>7.91</v>
       </c>
-      <c r="F71" s="8" t="inlineStr">
+      <c r="F72" s="8" t="inlineStr">
         <is>
           <t>197-19-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="G72" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H71" s="8" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="10" t="inlineStr">
+      <c r="H72" s="8" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>PM112501</t>
         </is>
       </c>
-      <c r="B72" s="10" t="inlineStr">
+      <c r="B73" s="10" t="inlineStr">
         <is>
           <t>Permanent Marker</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D72" s="10" t="inlineStr">
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
         <is>
           <t>PM_THC14 : CBD1</t>
         </is>
       </c>
-      <c r="E72" s="12" t="n">
+      <c r="E73" s="12" t="n">
         <v>13.33</v>
       </c>
-      <c r="F72" s="10" t="inlineStr">
+      <c r="F73" s="10" t="inlineStr">
         <is>
           <t>ППК26030, 05.03.2026, UKIM</t>
         </is>
       </c>
-      <c r="G72" s="11" t="inlineStr">
+      <c r="G73" s="11" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H72" s="10" t="inlineStr">
+      <c r="H73" s="10" t="inlineStr">
         <is>
           <t>owner code THC12 infeasible for audited 13.33 — moved to THC14</t>
         </is>
       </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t>PM092501</t>
-        </is>
-      </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>Permanent Marker</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>II</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>PM_THC12 : CBD1</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="n">
-        <v>12.25</v>
-      </c>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>197-20-К/26, 07.08.2026, FARM</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H73" s="8" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>PM072501</t>
+          <t>PM092501</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
@@ -5674,82 +5719,78 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>PM_THC10 : CBD1</t>
+          <t>PM_THC12 : CBD1</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>10.01</v>
+        <v>12.25</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>ППК25368, 28.11.2025, UKIM</t>
+          <t>197-20-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H74" s="8" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>PUM102501</t>
+          <t>PM072501</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Pure Michigen</t>
+          <t>Permanent Marker</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>PUM_THC16 : CBD1</t>
+          <t>PM_THC10 : CBD1</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>15.63</v>
+        <v>10.01</v>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>owner-declared value</t>
+          <t>ППК25368, 28.11.2025, UKIM</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
         <is>
-          <t>declared value — no eCoA yet, grade provisional until tested</t>
+          <t>code assigned by value (batch not on the tranche list)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>SCR022601</t>
+          <t>PUM102501</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Scrambler</t>
+          <t>Pure Michigen</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
@@ -5759,32 +5800,32 @@
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>SCR_THC22 : CBD1</t>
+          <t>PUM_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>21.92</v>
+        <v>15.63</v>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>ППК26116, 06.07.2026, UKIM</t>
+          <t>owner-declared value</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
+          <t>declared value — no eCoA yet, grade provisional until tested</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>SCR012601</t>
+          <t>SCR022601</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
@@ -5794,20 +5835,20 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>SCR_THC18 : CBD1</t>
+          <t>SCR_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>18.07</v>
+        <v>21.92</v>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>owner-declared value</t>
+          <t>ППК26116, 06.07.2026, UKIM</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -5817,14 +5858,14 @@
       </c>
       <c r="H77" s="8" t="inlineStr">
         <is>
-          <t>declared value — no eCoA yet, grade provisional until tested</t>
+          <t>code assigned by value (batch not on the tranche list)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>SCR012603</t>
+          <t>SCR012601</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
@@ -5843,24 +5884,28 @@
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>17.84</v>
+        <v>18.07</v>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>197-21-К/26, 07.08.2026, FARM</t>
+          <t>owner-declared value</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H78" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>declared value — no eCoA yet, grade provisional until tested</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>SCR112501</t>
+          <t>SCR012603</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
@@ -5879,11 +5924,11 @@
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>17.13</v>
+        <v>17.84</v>
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>ППК26069, 11.05.2026, UKIM</t>
+          <t>197-21-К/26, 07.08.2026, FARM</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -5896,47 +5941,43 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>SJ102501</t>
+          <t>SCR112501</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Sleepy Joy</t>
+          <t>Scrambler</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>SJ_THC12 : CBD1</t>
+          <t>SCR_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E80" s="6" t="n">
-        <v>11.2</v>
+        <v>17.13</v>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>051-3-K/26, 04.03.2026, FARM</t>
+          <t>ППК26069, 11.05.2026, UKIM</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H80" s="8" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>SJ092501</t>
+          <t>SJ102501</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
@@ -5946,33 +5987,37 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>SJ_THC10 : CBD1</t>
+          <t>SJ_THC12 : CBD1</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>10.96</v>
+        <v>11.2</v>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>ППК26006, 21.01.2026, UKIM</t>
+          <t>051-3-K/26, 04.03.2026, FARM</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H81" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>code assigned by value (batch not on the tranche list)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>SJ112501</t>
+          <t>SJ092501</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
@@ -5991,51 +6036,47 @@
         </is>
       </c>
       <c r="E82" s="6" t="n">
-        <v>9.199999999999999</v>
+        <v>10.96</v>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>051-2-K/26, 04.03.2026, FARM</t>
+          <t>ППК26006, 21.01.2026, UKIM</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H82" s="8" t="inlineStr">
-        <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>WED102501</t>
+          <t>SJ112501</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Wedding Cake</t>
+          <t>Sleepy Joy</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>WED_THC22 : CBD1</t>
+          <t>SJ_THC10 : CBD1</t>
         </is>
       </c>
       <c r="E83" s="6" t="n">
-        <v>22.05</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>owner-declared value</t>
+          <t>051-2-K/26, 04.03.2026, FARM</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -6045,19 +6086,19 @@
       </c>
       <c r="H83" s="8" t="inlineStr">
         <is>
-          <t>declared value — no eCoA yet, grade provisional until tested</t>
+          <t>code assigned by value (batch not on the tranche list)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>WC072501</t>
+          <t>WED102501</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Wedding Crasher</t>
+          <t>Wedding Cake</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -6067,15 +6108,15 @@
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>WC_THC22 : CBD1</t>
+          <t>WED_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E84" s="6" t="n">
-        <v>22.11</v>
+        <v>22.05</v>
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>ППК25369, 28.11.2025, UKIM</t>
+          <t>owner-declared value</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -6085,45 +6126,85 @@
       </c>
       <c r="H84" s="8" t="inlineStr">
         <is>
-          <t>code assigned by value (batch not on the tranche list)</t>
+          <t>declared value — no eCoA yet, grade provisional until tested</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
+          <t>WC072501</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Wedding Crasher</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>WC_THC22 : CBD1</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>22.11</v>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>ППК25369, 28.11.2025, UKIM</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>code assigned by value (batch not on the tranche list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
           <t>WC082501</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B86" s="8" t="inlineStr">
         <is>
           <t>Wedding Crasher</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D85" s="8" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
         <is>
           <t>WC_THC22 : CBD1</t>
         </is>
       </c>
-      <c r="E85" s="6" t="n">
+      <c r="E86" s="6" t="n">
         <v>21.67</v>
       </c>
-      <c r="F85" s="8" t="inlineStr">
+      <c r="F86" s="8" t="inlineStr">
         <is>
           <t>ППК26001, 21.01.2026, UKIM</t>
         </is>
       </c>
-      <c r="G85" s="5" t="inlineStr">
+      <c r="G86" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H85" s="8" t="inlineStr"/>
+      <c r="H86" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6136,7 +6217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6200,88 +6281,88 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ODD-nominal fallback (management rule, 27.08.2026): an isolated result that no even nominal can hold within ±10% (the even ladder has dead zones at 6.61–7.19 and 8.81–8.99) takes the adjacent ODD whole-number nominal instead, formed without overlap against the neighbouring ranges. With this fallback every result above ≈5.0% THC is always placeable (for any value v, at least one whole number lies between v/1.1 and v/0.9 once v ≥ 5).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>FLAGS</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Graps &amp; Creme / GRC102501/1: 7.05 fits no even nominal (even-ladder dead zone) -&gt; ODD fallback THC7 [6.30-7.70]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Permanent Marker / PM112501: owner code THC12 infeasible for 13.33 (max window 10.80-13.20) -&gt; THC14</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>EXCEPTIONS</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Graps &amp; Creme / GRC102501/1: 7.05 (declared (no eCoA yet)) fits NO even nominal within +/-10% — dead zone, excluded pending re-test</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>none — the odd-nominal fallback (rule 5) resolves all former dead-zone cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>OPEN VERIFICATIONS CARRIED OVER</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>BSS052501: 20.39 (PP QCCoA 001v02) vs 20.47 on the owner sheet (unreadable NGP scan) — grade THC20 holds under either value; paper check pending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>OMP1024_01: 15.38 correction (cert ППК25117 prints 1.58 — printing anomaly) — VERIFY ON PAPER ORIGINAL; grade THC16 assumes 15.38.</t>
-        </is>
-      </c>
+      <c r="B15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -6291,7 +6372,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>GG1024_02: 15.95 correction (cert ППК25140 prints 15.59) — VERIFY ON PAPER ORIGINAL; grade THC16 holds under either value.</t>
+          <t>BSS052501: 20.39 (PP QCCoA 001v02) vs 20.47 on the owner sheet (unreadable NGP scan) — grade THC20 holds under either value; paper check pending.</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6384,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GP062501: PP cert prints 24.89 vs owner sheet 22.89 — grade THC24 holds under either value.</t>
+          <t>OMP1024_01: 15.38 correction (cert ППК25117 prints 1.58 — printing anomaly) — VERIFY ON PAPER ORIGINAL; grade THC16 assumes 15.38.</t>
         </is>
       </c>
     </row>
@@ -6315,7 +6396,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>J31122501 graded on the machine-trimmed CoQ-forming preparation (21.84, CoQ-PP-2026-0054); the hand-trimmed 19.84 result is experimental only.</t>
+          <t>GG1024_02: 15.95 correction (cert ППК25140 prints 15.59) — VERIFY ON PAPER ORIGINAL; grade THC16 holds under either value.</t>
         </is>
       </c>
     </row>
@@ -6326,6 +6407,30 @@
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>GP062501: PP cert prints 24.89 vs owner sheet 22.89 — grade THC24 holds under either value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>J31122501 graded on the machine-trimmed CoQ-forming preparation (21.84, CoQ-PP-2026-0054); the hand-trimmed 19.84 result is experimental only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Batches on declared values (no eCoA yet): ACC102501, CC012603, CF102501, JD012603/01, PUM102501 (T2 re-analysis sampled 12.08.2026, results pending), SCR012601, WED102501, JD022601, GRC102501/1, P160012, P160022, P160032 — their grades are provisional.</t>
         </is>

</xml_diff>

<commit_message>
Contiguity rule: gapless grade ladders with reserve grades; retest anchors codified
Two management rule additions (27.08.2026):
- Retest results are the CoQ-forming anchors: grades are designed on the
  latest (retest) value per batch; superseded pre-retest results are out
  of specification scope.
- Contiguity from the top grade down: consecutive ranges join without gap
  or overlap. Five RESERVE grades (spec-defined, no current batch) inserted
  where batch-bearing grades cannot join directly: CJ THC18+THC16,
  CC THC16, FB THC16, JD THC18, OPM THC12. Sole exception below 10% THC
  where the even ladder cannot join: GRC uncovered zone 7.71-10.79 above
  the THC7 floater, OPM 8.81-8.99 between THC10 and THC8.

24 strains, 58 grades (53 batch-bearing + 5 reserve), 85 batches placed;
contiguity, caps, nominal-inside and batch-containment all assert-verified.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/potency_study/ImB_Potency_Grade_Ranges.xlsx
+++ b/deliverables/potency_study/ImB_Potency_Grade_Ranges.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -812,7 +812,7 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K9" s="8" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="J10" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -933,17 +933,17 @@
         <v>20</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>18</v>
+        <v>18.01</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>20</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>CJ_THC14 : CBD1</t>
+          <t>CJ_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -971,74 +971,66 @@
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>12.6</v>
+        <v>16.2</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>15.4</v>
+        <v>18</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>1.8</v>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>RESERVE (contiguity bridge)</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>CJ052501/02 14.93</t>
+          <t>— reserve grade (no current batch)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Cash Cow</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
+      <c r="A14" s="8" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr"/>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>CC_THC18 : CBD1</t>
+          <t>CJ_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_CC-I</t>
+          <t>QCSP_001_CJ-V</t>
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>16.2</v>
+        <v>14.94</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>19.8</v>
+        <v>16.19</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>1.25</v>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>RESERVE (contiguity bridge)</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>CC012601/1 17.67</t>
+          <t>— reserve grade (no current batch)</t>
         </is>
       </c>
     </row>
@@ -1047,17 +1039,17 @@
       <c r="B15" s="5" t="inlineStr"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>VI</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>CC_THC14 : CBD1</t>
+          <t>CJ_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_CC-II</t>
+          <t>QCSP_001_CJ-VI</t>
         </is>
       </c>
       <c r="F15" s="6" t="n">
@@ -1067,379 +1059,379 @@
         <v>12.6</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>15.4</v>
+        <v>14.93</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
+        <v>2.33</v>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>CJ052501/02 14.93</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Cash Cow</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>CC_THC18 : CBD1</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_CC-I</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>CC012601/1 17.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>CC_THC16 : CBD1</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_CC-II</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>RESERVE (contiguity bridge)</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>— reserve grade (no current batch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>CC_THC14 : CBD1</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_CC-III</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>14.39</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>CC112501 13.35</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr"/>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>III</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>CC_THC12 : CBD1</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_CC-III</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_CC-IV</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G19" s="6" t="n">
         <v>10.8</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H19" s="6" t="n">
         <v>12.59</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I19" s="6" t="n">
         <v>1.79</v>
       </c>
-      <c r="J16" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>CC012603 12.32</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Chem Flyer</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>CF</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>CF_THC10 : CBD1</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_CF-I</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F20" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G20" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="H20" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="I20" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
         <is>
           <t>CF102501 9.83</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Clemosa a bud</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>CLE</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>CLE_THC8 : CBD1</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_CLE-I</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F21" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G21" s="6" t="n">
         <v>7.2</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H21" s="6" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I21" s="6" t="n">
         <v>1.6</v>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K18" s="8" t="inlineStr">
+      <c r="K21" s="8" t="inlineStr">
         <is>
           <t>CLE072501 8.02</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Fat Bastard</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>FB</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>FB_THC20 : CBD1</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_FB-I</t>
         </is>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F22" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G22" s="6" t="n">
         <v>18.87</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H22" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I22" s="6" t="n">
         <v>3.13</v>
       </c>
-      <c r="J19" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>FB012603 20.83</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>FB_THC18 : CBD1</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_FB-II</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>18.86</v>
-      </c>
-      <c r="I20" s="6" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="J20" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>FB012602 18.86, FB012603V 18.29, FB112501 16.69</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr"/>
-      <c r="B21" s="5" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>III</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>FB_THC14 : CBD1</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_FB-III</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="I21" s="6" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>FB012601/1 14.68</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>IV</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>FB_THC12 : CBD1</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_FB-IV</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="H22" s="6" t="n">
-        <v>12.59</v>
-      </c>
-      <c r="I22" s="6" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>FB032601 12.39</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Gorilla Glue</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>GG</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>GG_THC18 : CBD1</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_GG-I</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
         <v>18</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>16.71</v>
+        <v>16.2</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>19.8</v>
+        <v>18.86</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>3.09</v>
+        <v>2.66</v>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>GG032601 18.98, GG1024_01 18.67, GG112501 17.94</t>
+          <t>FB012602 18.86, FB012603V 18.29, FB112501 16.69</t>
         </is>
       </c>
     </row>
@@ -1448,39 +1440,39 @@
       <c r="B24" s="5" t="inlineStr"/>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>GG_THC16 : CBD1</t>
+          <t>FB_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GG-II</t>
+          <t>QCSP_001_FB-III</t>
         </is>
       </c>
       <c r="F24" s="6" t="n">
         <v>16</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>14.4</v>
+        <v>14.69</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>16.7</v>
+        <v>16.19</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>2.3</v>
+        <v>1.5</v>
       </c>
       <c r="J24" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>RESERVE (contiguity bridge)</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>GG012603 16.70, GG1024_02 15.95, GG012601 15.35</t>
+          <t>— reserve grade (no current batch)</t>
         </is>
       </c>
     </row>
@@ -1489,17 +1481,17 @@
       <c r="B25" s="5" t="inlineStr"/>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>GG_THC14 : CBD1</t>
+          <t>FB_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GG-III</t>
+          <t>QCSP_001_FB-IV</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
@@ -1509,109 +1501,109 @@
         <v>12.6</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>14.39</v>
+        <v>14.68</v>
       </c>
       <c r="I25" s="6" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>FB012601/1 14.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>FB_THC12 : CBD1</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_FB-V</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>12.59</v>
+      </c>
+      <c r="I26" s="6" t="n">
         <v>1.79</v>
       </c>
-      <c r="J25" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>GG1024 13.34</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Grape Pie</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>GP</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>FB032601 12.39</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Gorilla Glue</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>GP_THC24 : CBD1</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_GP-I</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="G26" s="6" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="H26" s="6" t="n">
-        <v>26.4</v>
-      </c>
-      <c r="I26" s="6" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>P160012 26.32, GP092501 25.73, P160022 25.72, GP0824_03 25.45, GP062501 24.89, P160032 24.78, GP0824_02 22.61</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>II</t>
-        </is>
-      </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>GP_THC20 : CBD1</t>
+          <t>GG_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GP-II</t>
+          <t>QCSP_001_GG-I</t>
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>18.53</v>
+        <v>16.71</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>21.59</v>
+        <v>19.8</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>3.06</v>
+        <v>3.09</v>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>GP072501/1 21.36, GP082501/1 21.29, GP0824_01 20.79, GP072501/2 19.81</t>
+          <t>GG032601 18.98, GG1024_01 18.67, GG112501 17.94</t>
         </is>
       </c>
     </row>
@@ -1620,39 +1612,39 @@
       <c r="B28" s="5" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>GP_THC18 : CBD1</t>
+          <t>GG_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GP-III</t>
+          <t>QCSP_001_GG-II</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>18.52</v>
+        <v>16.7</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2.32</v>
+        <v>2.3</v>
       </c>
       <c r="J28" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>GP052501 18.52</t>
+          <t>GG012603 16.70, GG1024_02 15.95, GG012601 15.35</t>
         </is>
       </c>
     </row>
@@ -1661,51 +1653,51 @@
       <c r="B29" s="5" t="inlineStr"/>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>GP_THC16 : CBD1</t>
+          <t>GG_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GP-IV</t>
+          <t>QCSP_001_GG-III</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>14.4</v>
+        <v>12.6</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>16.19</v>
+        <v>14.39</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>1.79</v>
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>GP082501/2 15.70</t>
+          <t>GG1024 13.34</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Graps &amp; Creme</t>
+          <t>Grape Pie</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>GRC</t>
+          <t>GP</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -1715,25 +1707,25 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>GRC_THC12 : CBD1</t>
+          <t>GP_THC24 : CBD1</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GRC-I</t>
+          <t>QCSP_001_GP-I</t>
         </is>
       </c>
       <c r="F30" s="6" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>10.8</v>
+        <v>21.6</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>13.2</v>
+        <v>26.4</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -1742,7 +1734,7 @@
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>GRC102501/2 11.53</t>
+          <t>P160012 26.32, GP092501 25.73, P160022 25.72, GP0824_03 25.45, GP062501 24.89, P160032 24.78, GP0824_02 22.61</t>
         </is>
       </c>
     </row>
@@ -1756,83 +1748,75 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>GRC_THC7 : CBD1</t>
+          <t>GP_THC20 : CBD1</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_GRC-II</t>
+          <t>QCSP_001_GP-II</t>
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>6.3</v>
+        <v>18.53</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>7.7</v>
+        <v>21.59</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10% — ODD nominal (fallback rule 5)</t>
+        <v>3.06</v>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>GRC102501/1 7.05</t>
+          <t>GP072501/1 21.36, GP082501/1 21.29, GP0824_01 20.79, GP072501/2 19.81</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>High Pro Amnesia</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>HPA</t>
-        </is>
-      </c>
+      <c r="A32" s="8" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr"/>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>HPA_THC22 : CBD1</t>
+          <t>GP_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_HPA-I</t>
+          <t>QCSP_001_GP-III</t>
         </is>
       </c>
       <c r="F32" s="6" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>19.8</v>
+        <v>16.2</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>24.2</v>
+        <v>18.52</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>2.32</v>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>HPA1024_01 21.61, HPA052501 20.39</t>
+          <t>GP052501 18.52</t>
         </is>
       </c>
     </row>
@@ -1841,51 +1825,51 @@
       <c r="B33" s="5" t="inlineStr"/>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>HPA_THC18 : CBD1</t>
+          <t>GP_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_HPA-II</t>
+          <t>QCSP_001_GP-IV</t>
         </is>
       </c>
       <c r="F33" s="6" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>19.79</v>
+        <v>16.19</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>3.59</v>
+        <v>1.79</v>
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>HPA1024 17.31</t>
+          <t>GP082501/2 15.70</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Jelly Donutz</t>
+          <t>Graps &amp; Creme</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>GRC</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -1895,25 +1879,25 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>JD_THC20 : CBD1</t>
+          <t>GRC_THC12 : CBD1</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_JD-I</t>
+          <t>QCSP_001_GRC-I</t>
         </is>
       </c>
       <c r="F34" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>18</v>
+        <v>10.8</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>22</v>
+        <v>13.2</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
@@ -1922,7 +1906,7 @@
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>JD012603/02 20.54, JD112501 20.32, JD022601 18.58, JD012601 18.16</t>
+          <t>GRC102501/2 11.53</t>
         </is>
       </c>
     </row>
@@ -1936,46 +1920,46 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>JD_THC16 : CBD1</t>
+          <t>GRC_THC7 : CBD1</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_JD-II</t>
+          <t>QCSP_001_GRC-II</t>
         </is>
       </c>
       <c r="F35" s="6" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>14.4</v>
+        <v>6.3</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>17.6</v>
+        <v>7.7</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>3.2</v>
+        <v>1.4</v>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>FULL ±10%</t>
+          <t>FULL ±10% — ODD nominal (fallback rule 5)</t>
         </is>
       </c>
       <c r="K35" s="8" t="inlineStr">
         <is>
-          <t>JD012603/01 16.71, JD012603/02V 15.16</t>
+          <t>GRC102501/1 7.05</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Jokerz 31</t>
+          <t>High Pro Amnesia</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>J31</t>
+          <t>HPA</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -1985,12 +1969,12 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>J31_THC22 : CBD1</t>
+          <t>HPA_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_J31-I</t>
+          <t>QCSP_001_HPA-I</t>
         </is>
       </c>
       <c r="F36" s="6" t="n">
@@ -2012,7 +1996,7 @@
       </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>J31122501 21.84, J31112501 20.21</t>
+          <t>HPA1024_01 21.61, HPA052501 20.39</t>
         </is>
       </c>
     </row>
@@ -2026,12 +2010,12 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>J31_THC18 : CBD1</t>
+          <t>HPA_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_J31-II</t>
+          <t>QCSP_001_HPA-II</t>
         </is>
       </c>
       <c r="F37" s="6" t="n">
@@ -2048,24 +2032,24 @@
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K37" s="8" t="inlineStr">
         <is>
-          <t>J31102501 17.32</t>
+          <t>HPA1024 17.31</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Kush Crasher</t>
+          <t>Jelly Donutz</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -2075,83 +2059,75 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>KC_THC18 : CBD1</t>
+          <t>JD_THC20 : CBD1</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_KC-I</t>
+          <t>QCSP_001_JD-I</t>
         </is>
       </c>
       <c r="F38" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>16.2</v>
+        <v>18.01</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>19.8</v>
+        <v>22</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="J38" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>3.99</v>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K38" s="8" t="inlineStr">
         <is>
-          <t>KC102501 17.04</t>
+          <t>JD012603/02 20.54, JD112501 20.32, JD022601 18.58, JD012601 18.16</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Motor Breath</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
+      <c r="A39" s="8" t="inlineStr"/>
+      <c r="B39" s="5" t="inlineStr"/>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>MB_THC18 : CBD1</t>
+          <t>JD_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_MB-I</t>
+          <t>QCSP_001_JD-II</t>
         </is>
       </c>
       <c r="F39" s="6" t="n">
         <v>18</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>16.83</v>
+        <v>16.72</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>19.8</v>
+        <v>18</v>
       </c>
       <c r="I39" s="6" t="n">
-        <v>2.97</v>
+        <v>1.28</v>
       </c>
       <c r="J39" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>RESERVE (contiguity bridge)</t>
         </is>
       </c>
       <c r="K39" s="8" t="inlineStr">
         <is>
-          <t>MB0824_04 18.67</t>
+          <t>— reserve grade (no current batch)</t>
         </is>
       </c>
     </row>
@@ -2160,17 +2136,17 @@
       <c r="B40" s="5" t="inlineStr"/>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>MB_THC16 : CBD1</t>
+          <t>JD_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_MB-II</t>
+          <t>QCSP_001_JD-III</t>
         </is>
       </c>
       <c r="F40" s="6" t="n">
@@ -2180,31 +2156,31 @@
         <v>14.4</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>16.82</v>
+        <v>16.71</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>2.42</v>
+        <v>2.31</v>
       </c>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>MB0824_05 16.82</t>
+          <t>JD012603/01 16.71, JD012603/02V 15.16</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Orange Punch Mimosa</t>
+          <t>Jokerz 31</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>OPM</t>
+          <t>J31</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2214,12 +2190,12 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC22 : CBD1</t>
+          <t>J31_THC22 : CBD1</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-I</t>
+          <t>QCSP_001_J31-I</t>
         </is>
       </c>
       <c r="F41" s="6" t="n">
@@ -2241,7 +2217,7 @@
       </c>
       <c r="K41" s="8" t="inlineStr">
         <is>
-          <t>OPM1024 20.03</t>
+          <t>J31122501 21.84, J31112501 20.21</t>
         </is>
       </c>
     </row>
@@ -2255,116 +2231,132 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC18 : CBD1</t>
+          <t>J31_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-II</t>
+          <t>QCSP_001_J31-II</t>
         </is>
       </c>
       <c r="F42" s="6" t="n">
         <v>18</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>16.56</v>
+        <v>16.2</v>
       </c>
       <c r="H42" s="6" t="n">
         <v>19.79</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>3.23</v>
+        <v>3.59</v>
       </c>
       <c r="J42" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>OPM1024_02 18.04</t>
+          <t>J31102501 17.32</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr"/>
-      <c r="B43" s="5" t="inlineStr"/>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Kush Crasher</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>KC</t>
+        </is>
+      </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC16 : CBD1</t>
+          <t>KC_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-III</t>
+          <t>QCSP_001_KC-I</t>
         </is>
       </c>
       <c r="F43" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>14.4</v>
+        <v>16.2</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>16.55</v>
+        <v>19.8</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="J43" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
+        <v>3.6</v>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
         </is>
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>OPM1024_03 16.55, OMP1024_01 15.38</t>
+          <t>KC102501 17.04</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr"/>
-      <c r="B44" s="5" t="inlineStr"/>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Motor Breath</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC14 : CBD1</t>
+          <t>MB_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-IV</t>
+          <t>QCSP_001_MB-I</t>
         </is>
       </c>
       <c r="F44" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>12.6</v>
+        <v>16.83</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>14.39</v>
+        <v>19.8</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>1.79</v>
+        <v>2.97</v>
       </c>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K44" s="8" t="inlineStr">
         <is>
-          <t>OPM052501 14.16</t>
+          <t>MB0824_04 18.67</t>
         </is>
       </c>
     </row>
@@ -2373,129 +2365,129 @@
       <c r="B45" s="5" t="inlineStr"/>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>OPM_THC10 : CBD1</t>
+          <t>MB_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_OPM-V</t>
+          <t>QCSP_001_MB-II</t>
         </is>
       </c>
       <c r="F45" s="6" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>9</v>
+        <v>14.4</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>11</v>
+        <v>16.82</v>
       </c>
       <c r="I45" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J45" s="7" t="inlineStr">
+        <v>2.42</v>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K45" s="8" t="inlineStr">
+        <is>
+          <t>MB0824_05 16.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Orange Punch Mimosa</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>OPM</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>OPM_THC22 : CBD1</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_OPM-I</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K45" s="8" t="inlineStr">
-        <is>
-          <t>OPM092501 9.43</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr"/>
-      <c r="B46" s="5" t="inlineStr"/>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>VI</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>OPM_THC8 : CBD1</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_OPM-VI</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="G46" s="6" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="H46" s="6" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="I46" s="6" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="J46" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
-        </is>
-      </c>
       <c r="K46" s="8" t="inlineStr">
         <is>
-          <t>OPM112501 8.00, OPM122501 7.91</t>
+          <t>OPM1024 20.03</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>Permanent Marker</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
+      <c r="A47" s="8" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr"/>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>PM_THC14 : CBD1</t>
+          <t>OPM_THC18 : CBD1</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_PM-I</t>
+          <t>QCSP_001_OPM-II</t>
         </is>
       </c>
       <c r="F47" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>12.6</v>
+        <v>16.56</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>15.4</v>
+        <v>19.79</v>
       </c>
       <c r="I47" s="6" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="J47" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>3.23</v>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K47" s="8" t="inlineStr">
         <is>
-          <t>PM112501 13.33</t>
+          <t>OPM1024_02 18.04</t>
         </is>
       </c>
     </row>
@@ -2504,39 +2496,39 @@
       <c r="B48" s="5" t="inlineStr"/>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>PM_THC12 : CBD1</t>
+          <t>OPM_THC16 : CBD1</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_PM-II</t>
+          <t>QCSP_001_OPM-III</t>
         </is>
       </c>
       <c r="F48" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>10.8</v>
+        <v>14.4</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>12.59</v>
+        <v>16.55</v>
       </c>
       <c r="I48" s="6" t="n">
-        <v>1.79</v>
+        <v>2.15</v>
       </c>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K48" s="8" t="inlineStr">
         <is>
-          <t>PM092501 12.25</t>
+          <t>OPM1024_03 16.55, OMP1024_01 15.38</t>
         </is>
       </c>
     </row>
@@ -2545,137 +2537,121 @@
       <c r="B49" s="5" t="inlineStr"/>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>PM_THC10 : CBD1</t>
+          <t>OPM_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_PM-III</t>
+          <t>QCSP_001_OPM-IV</t>
         </is>
       </c>
       <c r="F49" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G49" s="6" t="n">
-        <v>9</v>
+        <v>12.6</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>10.79</v>
+        <v>14.39</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>1.79</v>
       </c>
       <c r="J49" s="9" t="inlineStr">
         <is>
-          <t>clipped (no-overlap rule)</t>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K49" s="8" t="inlineStr">
         <is>
-          <t>PM072501 10.01</t>
+          <t>OPM052501 14.16</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Pure Michigen</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>PUM</t>
-        </is>
-      </c>
+      <c r="A50" s="8" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr"/>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>PUM_THC16 : CBD1</t>
+          <t>OPM_THC12 : CBD1</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_PUM-I</t>
+          <t>QCSP_001_OPM-V</t>
         </is>
       </c>
       <c r="F50" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>14.4</v>
+        <v>10.8</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>17.6</v>
+        <v>12.59</v>
       </c>
       <c r="I50" s="6" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="J50" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>1.79</v>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>RESERVE (contiguity bridge)</t>
         </is>
       </c>
       <c r="K50" s="8" t="inlineStr">
         <is>
-          <t>PUM102501 15.63</t>
+          <t>— reserve grade (no current batch)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Scrambler</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>SCR</t>
-        </is>
-      </c>
+      <c r="A51" s="8" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr"/>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>VI</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>SCR_THC22 : CBD1</t>
+          <t>OPM_THC10 : CBD1</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_SCR-I</t>
+          <t>QCSP_001_OPM-VI</t>
         </is>
       </c>
       <c r="F51" s="6" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G51" s="6" t="n">
-        <v>19.8</v>
+        <v>9</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>24.2</v>
+        <v>10.79</v>
       </c>
       <c r="I51" s="6" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J51" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>1.79</v>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K51" s="8" t="inlineStr">
         <is>
-          <t>SCR022601 21.92</t>
+          <t>OPM092501 9.43</t>
         </is>
       </c>
     </row>
@@ -2684,51 +2660,51 @@
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>VII</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>SCR_THC18 : CBD1</t>
+          <t>OPM_THC8 : CBD1</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_SCR-II</t>
+          <t>QCSP_001_OPM-VII</t>
         </is>
       </c>
       <c r="F52" s="6" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G52" s="6" t="n">
-        <v>16.2</v>
+        <v>7.2</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>19.79</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I52" s="6" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="J52" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
+        <v>1.6</v>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
         </is>
       </c>
       <c r="K52" s="8" t="inlineStr">
         <is>
-          <t>SCR012601 18.07, SCR012603 17.84, SCR112501 17.13</t>
+          <t>OPM112501 8.00, OPM122501 7.91</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Sleepy Joy</t>
+          <t>Permanent Marker</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -2738,34 +2714,34 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>SJ_THC12 : CBD1</t>
+          <t>PM_THC14 : CBD1</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_SJ-I</t>
+          <t>QCSP_001_PM-I</t>
         </is>
       </c>
       <c r="F53" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>10.97</v>
+        <v>12.6</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>13.2</v>
+        <v>15.4</v>
       </c>
       <c r="I53" s="6" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="J53" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
+        <v>2.8</v>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
         </is>
       </c>
       <c r="K53" s="8" t="inlineStr">
         <is>
-          <t>SJ102501 11.20</t>
+          <t>PM112501 13.33</t>
         </is>
       </c>
     </row>
@@ -2779,130 +2755,400 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>SJ_THC10 : CBD1</t>
+          <t>PM_THC12 : CBD1</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>QCSP_001_SJ-II</t>
+          <t>QCSP_001_PM-II</t>
         </is>
       </c>
       <c r="F54" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>12.59</v>
+      </c>
+      <c r="I54" s="6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K54" s="8" t="inlineStr">
+        <is>
+          <t>PM092501 12.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr"/>
+      <c r="B55" s="5" t="inlineStr"/>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>PM_THC10 : CBD1</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_PM-III</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G54" s="6" t="n">
+      <c r="G55" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H54" s="6" t="n">
-        <v>10.96</v>
-      </c>
-      <c r="I54" s="6" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="J54" s="9" t="inlineStr">
-        <is>
-          <t>clipped (no-overlap rule)</t>
-        </is>
-      </c>
-      <c r="K54" s="8" t="inlineStr">
-        <is>
-          <t>SJ092501 10.96, SJ112501 9.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>Wedding Cake</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>WED</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>WED_THC22 : CBD1</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>QCSP_001_WED-I</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>19.8</v>
-      </c>
       <c r="H55" s="6" t="n">
-        <v>24.2</v>
+        <v>10.79</v>
       </c>
       <c r="I55" s="6" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J55" s="7" t="inlineStr">
-        <is>
-          <t>FULL ±10%</t>
+        <v>1.79</v>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
         </is>
       </c>
       <c r="K55" s="8" t="inlineStr">
         <is>
-          <t>WED102501 22.05</t>
+          <t>PM072501 10.01</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
+          <t>Pure Michigen</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>PUM</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>PUM_THC16 : CBD1</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_PUM-I</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K56" s="8" t="inlineStr">
+        <is>
+          <t>PUM102501 15.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Scrambler</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>SCR</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>SCR_THC22 : CBD1</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_SCR-I</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H57" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="I57" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K57" s="8" t="inlineStr">
+        <is>
+          <t>SCR022601 21.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr"/>
+      <c r="B58" s="5" t="inlineStr"/>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>SCR_THC18 : CBD1</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_SCR-II</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="I58" s="6" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K58" s="8" t="inlineStr">
+        <is>
+          <t>SCR012601 18.07, SCR012603 17.84, SCR112501 17.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Sleepy Joy</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>SJ</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>SJ_THC12 : CBD1</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_SJ-I</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="H59" s="6" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I59" s="6" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K59" s="8" t="inlineStr">
+        <is>
+          <t>SJ102501 11.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr"/>
+      <c r="B60" s="5" t="inlineStr"/>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>SJ_THC10 : CBD1</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_SJ-II</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G60" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H60" s="6" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="I60" s="6" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J60" s="9" t="inlineStr">
+        <is>
+          <t>clipped (contiguity rule)</t>
+        </is>
+      </c>
+      <c r="K60" s="8" t="inlineStr">
+        <is>
+          <t>SJ092501 10.96, SJ112501 9.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Wedding Cake</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>WED</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>WED_THC22 : CBD1</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>QCSP_001_WED-I</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H61" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="I61" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>FULL ±10%</t>
+        </is>
+      </c>
+      <c r="K61" s="8" t="inlineStr">
+        <is>
+          <t>WED102501 22.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
           <t>Wedding Crasher</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>WC_THC22 : CBD1</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>QCSP_001_WC-I</t>
         </is>
       </c>
-      <c r="F56" s="6" t="n">
+      <c r="F62" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G56" s="6" t="n">
+      <c r="G62" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="H56" s="6" t="n">
+      <c r="H62" s="6" t="n">
         <v>24.2</v>
       </c>
-      <c r="I56" s="6" t="n">
+      <c r="I62" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="J56" s="7" t="inlineStr">
+      <c r="J62" s="7" t="inlineStr">
         <is>
           <t>FULL ±10%</t>
         </is>
       </c>
-      <c r="K56" s="8" t="inlineStr">
+      <c r="K62" s="8" t="inlineStr">
         <is>
           <t>WC072501 22.11, WC082501 21.67</t>
         </is>
@@ -3515,7 +3761,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>VI</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -3595,7 +3841,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -3635,7 +3881,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -3907,7 +4153,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -3943,7 +4189,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -5079,7 +5325,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -5119,7 +5365,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -5567,7 +5813,7 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>VI</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
@@ -5603,7 +5849,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>VI</t>
+          <t>VII</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
@@ -5643,7 +5889,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>VI</t>
+          <t>VII</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
@@ -6217,7 +6463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6288,81 +6534,93 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ODD-nominal fallback (management rule, 27.08.2026): an isolated result that no even nominal can hold within ±10% (the even ladder has dead zones at 6.61–7.19 and 8.81–8.99) takes the adjacent ODD whole-number nominal instead, formed without overlap against the neighbouring ranges. With this fallback every result above ≈5.0% THC is always placeable (for any value v, at least one whole number lies between v/1.1 and v/0.9 once v ≥ 5).</t>
+          <t>Retest results are the CoQ-forming anchors (management rule, 27.08.2026): where a batch has a retest (Tranche 1 197-series of 07.08.2026, the April J31 retests, and the pending Tranche 2 re-analysis when it lands), the grade is designed on the retest value; superseded pre-retest results are out of specification scope.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Contiguity (management rule, 27.08.2026): from the top grade down, consecutive grade ranges join without gap or overlap (upper of the weaker = lower of the stronger minus 0.01). Where batch-bearing grades cannot join directly, RESERVE grades (spec-defined, no current batch) are inserted to close the span. Sole exception: below 10% THC, where the ladder mathematically cannot join, the lowest grade(s) may sit with a documented uncovered zone above them (GRC 7.71-10.79; OPM 8.81-8.99).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ODD-nominal fallback (management rule, 27.08.2026): an isolated result that no even nominal can hold within ±10% (the even ladder has dead zones at 6.61–7.19 and 8.81–8.99) takes the adjacent ODD whole-number nominal instead, formed without overlap against the neighbouring ranges. With this fallback every result above ≈5.0% THC is always placeable (for any value v, at least one whole number lies between v/1.1 and v/0.9 once v ≥ 5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
           <t>FLAGS</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Graps &amp; Creme / GRC102501/1: 7.05 fits no even nominal (even-ladder dead zone) -&gt; ODD fallback THC7 [6.30-7.70]</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Permanent Marker / PM112501: owner code THC12 infeasible for 13.33 (max window 10.80-13.20) -&gt; THC14</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>EXCEPTIONS</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>none — the odd-nominal fallback (rule 5) resolves all former dead-zone cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>OPEN VERIFICATIONS CARRIED OVER</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Graps &amp; Creme: uncovered zone 7.71-10.79 between THC12 and THC7 (sub-10% territory — even ladder cannot join; permitted per rule)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -6372,33 +6630,21 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>BSS052501: 20.39 (PP QCCoA 001v02) vs 20.47 on the owner sheet (unreadable NGP scan) — grade THC20 holds under either value; paper check pending.</t>
+          <t>Orange Punch Mimosa: uncovered zone 8.81-8.99 between THC10 and THC8 (sub-10% territory — even ladder cannot join; permitted per rule)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>OMP1024_01: 15.38 correction (cert ППК25117 prints 1.58 — printing anomaly) — VERIFY ON PAPER ORIGINAL; grade THC16 assumes 15.38.</t>
-        </is>
-      </c>
+      <c r="A17" s="14" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>GG1024_02: 15.95 correction (cert ППК25140 prints 15.59) — VERIFY ON PAPER ORIGINAL; grade THC16 holds under either value.</t>
-        </is>
-      </c>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>OPEN VERIFICATIONS CARRIED OVER</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
@@ -6408,7 +6654,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>GP062501: PP cert prints 24.89 vs owner sheet 22.89 — grade THC24 holds under either value.</t>
+          <t>BSS052501: 20.39 (PP QCCoA 001v02) vs 20.47 on the owner sheet (unreadable NGP scan) — grade THC20 holds under either value; paper check pending.</t>
         </is>
       </c>
     </row>
@@ -6420,7 +6666,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>J31122501 graded on the machine-trimmed CoQ-forming preparation (21.84, CoQ-PP-2026-0054); the hand-trimmed 19.84 result is experimental only.</t>
+          <t>OMP1024_01: 15.38 correction (cert ППК25117 prints 1.58 — printing anomaly) — VERIFY ON PAPER ORIGINAL; grade THC16 assumes 15.38.</t>
         </is>
       </c>
     </row>
@@ -6431,6 +6677,42 @@
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>GG1024_02: 15.95 correction (cert ППК25140 prints 15.59) — VERIFY ON PAPER ORIGINAL; grade THC16 holds under either value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>GP062501: PP cert prints 24.89 vs owner sheet 22.89 — grade THC24 holds under either value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>J31122501 graded on the machine-trimmed CoQ-forming preparation (21.84, CoQ-PP-2026-0054); the hand-trimmed 19.84 result is experimental only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Batches on declared values (no eCoA yet): ACC102501, CC012603, CF102501, JD012603/01, PUM102501 (T2 re-analysis sampled 12.08.2026, results pending), SCR012601, WED102501, JD022601, GRC102501/1, P160012, P160022, P160032 — their grades are provisional.</t>
         </is>

</xml_diff>